<commit_message>
updated main holder bom for 320
</commit_message>
<xml_diff>
--- a/accessories/cable-5/cable-5.xlsx
+++ b/accessories/cable-5/cable-5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\Battery-Lab-Hardware\accessories\cable-5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A27FCA7C-9D80-45C4-9234-73C9A83FDE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A4293A-B9B1-462D-AAD8-412DCD3847F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3090" windowWidth="21600" windowHeight="11295" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDAE7DA4-9528-4FC7-A320-70DA50473DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="bill_of_materials" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="77">
   <si>
     <t>Individual Cost</t>
   </si>
@@ -258,6 +258,15 @@
   </si>
   <si>
     <t>TERM BLADE FEMALE 14-18AWG SILV</t>
+  </si>
+  <si>
+    <t>Main Female Housing</t>
+  </si>
+  <si>
+    <t>A32500-0009</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/anderson-power-products-inc/A32500-0009/14833308?s=N4IgTCBcDaIIIGYwFYAMqC07UE4QF0BfIA</t>
   </si>
 </sst>
 </file>
@@ -866,27 +875,27 @@
       <c r="J2" s="2"/>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="19">
+      <c r="D3" s="23">
         <v>1</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="24">
         <v>19.18</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="24">
         <f>D3*E3</f>
         <v>19.18</v>
       </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="1" t="s">
+      <c r="G3" s="25"/>
+      <c r="H3" s="26" t="s">
         <v>15</v>
       </c>
       <c r="I3" s="1"/>
@@ -1176,7 +1185,7 @@
         <v>72.62</v>
       </c>
       <c r="F14" s="9">
-        <f t="shared" ref="F14:F17" si="3">D14*E14</f>
+        <f t="shared" ref="F14:F18" si="3">D14*E14</f>
         <v>72.62</v>
       </c>
       <c r="G14" s="5"/>
@@ -1264,14 +1273,29 @@
       <c r="I17" s="4"/>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="9"/>
+      <c r="A18" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D18" s="2">
+        <v>1</v>
+      </c>
+      <c r="E18" s="8">
+        <v>23.22</v>
+      </c>
+      <c r="F18" s="9">
+        <f t="shared" si="3"/>
+        <v>23.22</v>
+      </c>
       <c r="G18" s="5"/>
-      <c r="H18" s="3"/>
+      <c r="H18" s="3" t="s">
+        <v>76</v>
+      </c>
       <c r="I18" s="4"/>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1317,7 +1341,7 @@
       </c>
       <c r="F23" s="5">
         <f>SUM(F2:F22)</f>
-        <v>460.21999999999997</v>
+        <v>483.43999999999994</v>
       </c>
     </row>
   </sheetData>
@@ -1341,8 +1365,9 @@
     <hyperlink ref="H9" r:id="rId16" xr:uid="{0BF14A02-DB2B-44C8-ADFD-F6B888D0D1E2}"/>
     <hyperlink ref="H5" r:id="rId17" xr:uid="{D098FC55-60BA-44A1-88B5-F7A95F7F2234}"/>
     <hyperlink ref="H8" r:id="rId18" xr:uid="{E4B64C1A-2E26-4C6F-9252-C15670A96A6B}"/>
+    <hyperlink ref="H18" r:id="rId19" xr:uid="{BC482846-CA0B-4C8C-A6F1-3CDFDF09F63D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId19"/>
+  <pageSetup orientation="portrait" r:id="rId20"/>
 </worksheet>
 </file>
</xml_diff>